<commit_message>
📊 Horarios actualizados Línea 141 - 5063
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-10-11.xlsx
+++ b/data/horarios-141-2026-10-11.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:23:59</t>
+          <t>Última actualización: 11:14:06</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 9</t>
+          <t>Total filas: 18</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04:23:59</t>
+          <t>11:14:06</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>04:47</t>
+          <t>11:16</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>04:23:59</t>
+          <t>11:14:06</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>04:52</t>
+          <t>11:24</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>04:23:59</t>
+          <t>11:14:06</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>05:16</t>
+          <t>11:35</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>53</v>
+        <v>21</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>04:23:59</t>
+          <t>11:14:06</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>05:21</t>
+          <t>11:36</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>58</v>
+        <v>22</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>04:23:59</t>
+          <t>11:14:06</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>05:46</t>
+          <t>11:42</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>83</v>
+        <v>28</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,21 +598,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>04:23:59</t>
+          <t>11:14:06</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>05:47</t>
+          <t>11:45</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>84</v>
+        <v>31</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,21 +623,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>04:23:59</t>
+          <t>11:14:06</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06:00</t>
+          <t>11:54</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>97</v>
+        <v>40</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -648,21 +648,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>04:23:59</t>
+          <t>11:14:06</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06:08</t>
+          <t>11:55</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>105</v>
+        <v>41</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,23 +673,248 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>04:23:59</t>
+          <t>11:14:06</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>06:12</t>
+          <t>12:04</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>109</v>
+        <v>50</v>
       </c>
       <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>11:14:06</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>61</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>11:14:06</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>12:25</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>71</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>11:14:06</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>12:32</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>78</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>11:14:06</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>12:34</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>80</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>11:14:06</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>12:34</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>80</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>11:14:06</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>12:44</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>90</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>11:14:06</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>12:46</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>92</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>11:14:06</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>101</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>11:14:06</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>13:05</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>111</v>
+      </c>
+      <c r="E23" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -706,7 +931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -719,14 +944,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:23:59</t>
+          <t>Última actualización: 11:14:06</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -760,23 +985,73 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04:23:59</t>
+          <t>11:14:06</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>06:12</t>
+          <t>11:35</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>109</v>
+        <v>21</v>
       </c>
       <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>11:14:06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>31</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>11:14:06</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>101</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -793,7 +1068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -806,14 +1081,66 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:23:59</t>
+          <t>Última actualización: 11:14:06</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>11:14:06</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>11:23</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>9</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 5064
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-10-11.xlsx
+++ b/data/horarios-141-2026-10-11.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:14:06</t>
+          <t>Última actualización: 15:55:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 18</t>
+          <t>Total filas: 37</t>
         </is>
       </c>
     </row>
@@ -915,6 +915,481 @@
         <v>111</v>
       </c>
       <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>15:55:40</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>15:55</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>15:55:40</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>15:56</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>15:55:40</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>16:04</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>9</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>15:55:40</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>16:14</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>19</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>15:55:40</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>16:16</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>21</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>15:55:40</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>16:24</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>29</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>15:55:40</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>16:34</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>39</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>15:55:40</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>16:35</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>40</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>15:55:40</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>16:41</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>46</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>15:55:40</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>16:44</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>49</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>15:55:40</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>16:51</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>56</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>15:55:40</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>60</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>15:55:40</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>17:04</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>69</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>15:55:40</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>17:14</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>79</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>15:55:40</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>17:24</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>89</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>15:55:40</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>17:31</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>96</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>15:55:40</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>100</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>15:55:40</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>17:36</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>101</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>15:55:40</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>17:44</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>109</v>
+      </c>
+      <c r="E42" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -931,7 +1406,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -944,14 +1419,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:14:06</t>
+          <t>Última actualización: 15:55:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 5</t>
         </is>
       </c>
     </row>
@@ -1052,6 +1527,56 @@
         <v>101</v>
       </c>
       <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>15:55:40</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>17:14</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>79</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>15:55:40</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>17:44</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>109</v>
+      </c>
+      <c r="E10" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1068,7 +1593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1081,14 +1606,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:14:06</t>
+          <t>Última actualización: 15:55:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 4</t>
         </is>
       </c>
     </row>
@@ -1139,6 +1664,81 @@
         <v>9</v>
       </c>
       <c r="E6" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>15:55:40</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>16:02</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>7</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>15:55:40</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>16:29</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>34</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>15:55:40</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>17:22</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>87</v>
+      </c>
+      <c r="E9" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 5065
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-10-11.xlsx
+++ b/data/horarios-141-2026-10-11.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:55:40</t>
+          <t>Última actualización: 19:33:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 37</t>
+          <t>Total filas: 50</t>
         </is>
       </c>
     </row>
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -808,7 +808,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1390,6 +1390,331 @@
         <v>109</v>
       </c>
       <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>19:33:56</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>19:48</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>15</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>19:33:56</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>19:49</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>16</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>19:33:56</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>19:56</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>23</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>19:33:56</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>20:01</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>28</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>19:33:56</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>20:14</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>41</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>19:33:56</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>42</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>19:33:56</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>20:35</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>62</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>19:33:56</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>66</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>19:33:56</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>68</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>19:33:56</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>20:56</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>83</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>19:33:56</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>20:57</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>84</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>19:33:56</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>21:05</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>92</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>19:33:56</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>93</v>
+      </c>
+      <c r="E55" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1406,7 +1731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1419,14 +1744,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:55:40</t>
+          <t>Última actualización: 19:33:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 5</t>
+          <t>Total filas: 9</t>
         </is>
       </c>
     </row>
@@ -1577,6 +1902,106 @@
         <v>109</v>
       </c>
       <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>19:33:56</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>20:14</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>41</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>19:33:56</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>66</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>19:33:56</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>68</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>19:33:56</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>93</v>
+      </c>
+      <c r="E14" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1593,7 +2018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1606,14 +2031,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:55:40</t>
+          <t>Última actualización: 19:33:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 4</t>
+          <t>Total filas: 6</t>
         </is>
       </c>
     </row>
@@ -1739,6 +2164,56 @@
         <v>87</v>
       </c>
       <c r="E9" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>19:33:56</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>19:46</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>13</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>19:33:56</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>20:38</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>65</v>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 5066
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-10-11.xlsx
+++ b/data/horarios-141-2026-10-11.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:33:56</t>
+          <t>Última actualización: 22:41:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 50</t>
+          <t>Total filas: 56</t>
         </is>
       </c>
     </row>
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -808,7 +808,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1715,6 +1715,156 @@
         <v>93</v>
       </c>
       <c r="E55" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>22:41:42</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>22:43</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>2</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>22:41:42</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>22:55</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>14</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>22:41:42</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>23:06</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>25</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>22:41:42</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>23:28</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>47</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>22:41:42</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>23:40</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>59</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>22:41:42</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>23:49</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>68</v>
+      </c>
+      <c r="E61" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1731,7 +1881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1744,14 +1894,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:33:56</t>
+          <t>Última actualización: 22:41:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 9</t>
+          <t>Total filas: 11</t>
         </is>
       </c>
     </row>
@@ -2002,6 +2152,56 @@
         <v>93</v>
       </c>
       <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>22:41:42</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>23:28</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>47</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>22:41:42</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>23:40</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>59</v>
+      </c>
+      <c r="E16" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2031,7 +2231,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:33:56</t>
+          <t>Última actualización: 22:41:42</t>
         </is>
       </c>
     </row>

</xml_diff>